<commit_message>
updated tests for new postal formatting, updated test excel file to simulate data
</commit_message>
<xml_diff>
--- a/tests/excel-files/excel.xlsx
+++ b/tests/excel-files/excel.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1143" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1150" uniqueCount="200">
   <si>
     <t xml:space="preserve">Full Name</t>
   </si>
@@ -581,6 +581,9 @@
   </si>
   <si>
     <t xml:space="preserve">TX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4CN 3XL</t>
   </si>
   <si>
     <t xml:space="preserve">Joshua Daniel Morales</t>
@@ -3519,7 +3522,7 @@
         <v>74</v>
       </c>
       <c r="R40" s="1" t="n">
-        <v>12345</v>
+        <v>312</v>
       </c>
       <c r="S40" s="1" t="s">
         <v>31</v>
@@ -3584,7 +3587,7 @@
         <v>74</v>
       </c>
       <c r="R41" s="1" t="n">
-        <v>12345</v>
+        <v>312</v>
       </c>
       <c r="S41" s="1" t="s">
         <v>31</v>
@@ -3649,7 +3652,7 @@
         <v>74</v>
       </c>
       <c r="R42" s="1" t="n">
-        <v>12345</v>
+        <v>312</v>
       </c>
       <c r="S42" s="1" t="s">
         <v>31</v>
@@ -3714,7 +3717,7 @@
         <v>74</v>
       </c>
       <c r="R43" s="1" t="n">
-        <v>12345</v>
+        <v>312</v>
       </c>
       <c r="S43" s="1" t="s">
         <v>31</v>
@@ -3779,7 +3782,7 @@
         <v>74</v>
       </c>
       <c r="R44" s="1" t="n">
-        <v>12345</v>
+        <v>312</v>
       </c>
       <c r="S44" s="1" t="s">
         <v>31</v>
@@ -3844,7 +3847,7 @@
         <v>74</v>
       </c>
       <c r="R45" s="1" t="n">
-        <v>12345</v>
+        <v>312</v>
       </c>
       <c r="S45" s="1" t="s">
         <v>31</v>
@@ -3909,7 +3912,7 @@
         <v>74</v>
       </c>
       <c r="R46" s="1" t="n">
-        <v>12345</v>
+        <v>312</v>
       </c>
       <c r="S46" s="1" t="s">
         <v>31</v>
@@ -3974,7 +3977,7 @@
         <v>74</v>
       </c>
       <c r="R47" s="1" t="n">
-        <v>12345</v>
+        <v>312</v>
       </c>
       <c r="S47" s="1" t="s">
         <v>31</v>
@@ -4039,7 +4042,7 @@
         <v>74</v>
       </c>
       <c r="R48" s="1" t="n">
-        <v>12345</v>
+        <v>312</v>
       </c>
       <c r="S48" s="1" t="s">
         <v>31</v>
@@ -4104,7 +4107,7 @@
         <v>74</v>
       </c>
       <c r="R49" s="1" t="n">
-        <v>12345</v>
+        <v>312</v>
       </c>
       <c r="S49" s="1" t="s">
         <v>31</v>
@@ -4169,7 +4172,7 @@
         <v>74</v>
       </c>
       <c r="R50" s="1" t="n">
-        <v>12345</v>
+        <v>312</v>
       </c>
       <c r="S50" s="1" t="s">
         <v>31</v>
@@ -4624,7 +4627,7 @@
         <v>145</v>
       </c>
       <c r="R57" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S57" s="1" t="s">
         <v>31</v>
@@ -4689,7 +4692,7 @@
         <v>145</v>
       </c>
       <c r="R58" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S58" s="1" t="s">
         <v>31</v>
@@ -4754,7 +4757,7 @@
         <v>145</v>
       </c>
       <c r="R59" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S59" s="1" t="s">
         <v>31</v>
@@ -4819,7 +4822,7 @@
         <v>145</v>
       </c>
       <c r="R60" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S60" s="1" t="s">
         <v>31</v>
@@ -4884,7 +4887,7 @@
         <v>145</v>
       </c>
       <c r="R61" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S61" s="1" t="s">
         <v>31</v>
@@ -4949,7 +4952,7 @@
         <v>145</v>
       </c>
       <c r="R62" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S62" s="1" t="s">
         <v>31</v>
@@ -5014,7 +5017,7 @@
         <v>145</v>
       </c>
       <c r="R63" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S63" s="1" t="s">
         <v>31</v>
@@ -5079,7 +5082,7 @@
         <v>145</v>
       </c>
       <c r="R64" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S64" s="1" t="s">
         <v>31</v>
@@ -5144,7 +5147,7 @@
         <v>145</v>
       </c>
       <c r="R65" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S65" s="1" t="s">
         <v>31</v>
@@ -5209,7 +5212,7 @@
         <v>145</v>
       </c>
       <c r="R66" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S66" s="1" t="s">
         <v>31</v>
@@ -5274,7 +5277,7 @@
         <v>145</v>
       </c>
       <c r="R67" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S67" s="1" t="s">
         <v>31</v>
@@ -5339,7 +5342,7 @@
         <v>145</v>
       </c>
       <c r="R68" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S68" s="1" t="s">
         <v>31</v>
@@ -5404,7 +5407,7 @@
         <v>145</v>
       </c>
       <c r="R69" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S69" s="1" t="s">
         <v>31</v>
@@ -5469,7 +5472,7 @@
         <v>145</v>
       </c>
       <c r="R70" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S70" s="1" t="s">
         <v>31</v>
@@ -5534,7 +5537,7 @@
         <v>145</v>
       </c>
       <c r="R71" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S71" s="1" t="s">
         <v>31</v>
@@ -5599,7 +5602,7 @@
         <v>145</v>
       </c>
       <c r="R72" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S72" s="1" t="s">
         <v>31</v>
@@ -5664,7 +5667,7 @@
         <v>145</v>
       </c>
       <c r="R73" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S73" s="1" t="s">
         <v>31</v>
@@ -5729,7 +5732,7 @@
         <v>145</v>
       </c>
       <c r="R74" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S74" s="1" t="s">
         <v>31</v>
@@ -5794,7 +5797,7 @@
         <v>145</v>
       </c>
       <c r="R75" s="1" t="n">
-        <v>12345</v>
+        <v>4431</v>
       </c>
       <c r="S75" s="1" t="s">
         <v>31</v>
@@ -5858,8 +5861,8 @@
       <c r="Q76" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="R76" s="1" t="n">
-        <v>12345</v>
+      <c r="R76" s="1" t="s">
+        <v>187</v>
       </c>
       <c r="S76" s="1" t="s">
         <v>31</v>
@@ -5873,10 +5876,10 @@
     </row>
     <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>23</v>
@@ -5923,8 +5926,8 @@
       <c r="Q77" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="R77" s="1" t="n">
-        <v>12345</v>
+      <c r="R77" s="1" t="s">
+        <v>187</v>
       </c>
       <c r="S77" s="1" t="s">
         <v>31</v>
@@ -5938,10 +5941,10 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>23</v>
@@ -5988,8 +5991,8 @@
       <c r="Q78" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="R78" s="1" t="n">
-        <v>12345</v>
+      <c r="R78" s="1" t="s">
+        <v>187</v>
       </c>
       <c r="S78" s="1" t="s">
         <v>31</v>
@@ -6003,10 +6006,10 @@
     </row>
     <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>23</v>
@@ -6053,8 +6056,8 @@
       <c r="Q79" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="R79" s="1" t="n">
-        <v>12345</v>
+      <c r="R79" s="1" t="s">
+        <v>187</v>
       </c>
       <c r="S79" s="1" t="s">
         <v>31</v>
@@ -6068,10 +6071,10 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>23</v>
@@ -6118,8 +6121,8 @@
       <c r="Q80" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="R80" s="1" t="n">
-        <v>12345</v>
+      <c r="R80" s="1" t="s">
+        <v>187</v>
       </c>
       <c r="S80" s="1" t="s">
         <v>31</v>
@@ -6133,10 +6136,10 @@
     </row>
     <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>23</v>
@@ -6183,8 +6186,8 @@
       <c r="Q81" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="R81" s="1" t="n">
-        <v>12345</v>
+      <c r="R81" s="1" t="s">
+        <v>187</v>
       </c>
       <c r="S81" s="1" t="s">
         <v>31</v>
@@ -6198,10 +6201,10 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>23</v>
@@ -6248,8 +6251,8 @@
       <c r="Q82" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="R82" s="1" t="n">
-        <v>12345</v>
+      <c r="R82" s="1" t="s">
+        <v>187</v>
       </c>
       <c r="S82" s="1" t="s">
         <v>31</v>

</xml_diff>